<commit_message>
Modified Cible pour AA ACUR/GDL
</commit_message>
<xml_diff>
--- a/tests/Cible.xlsx
+++ b/tests/Cible.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MAYT8801\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mayt8801\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -1048,7 +1048,7 @@
         <v>0</v>
       </c>
       <c r="E34" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="18">
@@ -1065,7 +1065,7 @@
         <v>0</v>
       </c>
       <c r="E35" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="18">

</xml_diff>